<commit_message>
changed order of st7
</commit_message>
<xml_diff>
--- a/data/programa.xlsx
+++ b/data/programa.xlsx
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="E44" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F44" s="6" t="n">
         <v>35100</v>
@@ -2113,7 +2113,7 @@
         </is>
       </c>
       <c r="E45" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F45" s="6" t="n">
         <v>35855</v>
@@ -2156,7 +2156,7 @@
         </is>
       </c>
       <c r="E46" s="6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46" s="6" t="n">
         <v>35177</v>
@@ -4260,7 +4260,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21" ht="15.75" customHeight="1" s="8">
       <c r="A21" s="6" t="inlineStr">
         <is>

</xml_diff>